<commit_message>
Fixed COR yo look at it
</commit_message>
<xml_diff>
--- a/New_CenterOfRotation/Finite_COR/Data Files/C34_Data/Y_Z Data Model 15-C34.xlsx
+++ b/New_CenterOfRotation/Finite_COR/Data Files/C34_Data/Y_Z Data Model 15-C34.xlsx
@@ -4,7 +4,7 @@
   <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="0"/>
+    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet r:id="rId1" sheetId="1" name="4N"/>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="264" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="258" uniqueCount="15">
   <si>
     <t>Descriptions are [X,Y,Z] coords in the model. If a node is in the middle on the right, and top of C4, it would be [1,0,1] C4. Bottom would be [1,0,-1] C4</t>
   </si>
@@ -71,19 +71,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
@@ -150,7 +144,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="21">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
@@ -161,40 +155,40 @@
     <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="3" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="3" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
@@ -208,9 +202,6 @@
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -521,28 +512,28 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" style="17" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="21" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="21" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="20" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="20" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="4" max="4" style="19" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="5" max="5" style="17" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="21" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="21" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="20" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="20" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="8" max="8" style="19" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="9" max="9" style="17" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="21" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="21" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="20" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="20" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="12" max="12" style="19" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="13" max="13" style="17" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="14" max="14" style="21" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="15" max="15" style="21" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="14" max="14" style="20" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="15" max="15" style="20" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="16" max="16" style="19" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="17" max="17" style="17" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="18" max="18" style="21" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="19" max="19" style="21" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="18" max="18" style="20" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="19" max="19" style="20" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="20" max="20" style="19" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="21" max="21" style="17" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="22" max="22" style="21" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="23" max="23" style="21" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="22" max="22" style="20" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="23" max="23" style="20" width="13.576428571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
@@ -1012,7 +1003,7 @@
       <c r="N9" s="14">
         <v>1.40913</v>
       </c>
-      <c r="O9" s="20">
+      <c r="O9" s="3">
         <v>-0.0991855</v>
       </c>
       <c r="P9" s="11"/>
@@ -2087,28 +2078,28 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" style="17" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="21" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="21" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="20" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="20" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="4" max="4" style="19" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="5" max="5" style="17" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="21" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="21" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="20" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="20" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="8" max="8" style="19" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="9" max="9" style="17" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="21" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="21" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="20" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="20" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="12" max="12" style="19" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="13" max="13" style="17" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="14" max="14" style="21" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="15" max="15" style="21" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="14" max="14" style="20" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="15" max="15" style="20" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="16" max="16" style="19" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="17" max="17" style="17" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="18" max="18" style="21" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="19" max="19" style="21" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="18" max="18" style="20" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="19" max="19" style="20" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="20" max="20" style="19" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="21" max="21" style="17" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="22" max="22" style="21" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="23" max="23" style="21" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="22" max="22" style="20" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="23" max="23" style="20" width="13.576428571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="15">
@@ -2578,7 +2569,7 @@
       <c r="N9" s="14">
         <v>-2.35262</v>
       </c>
-      <c r="O9" s="20">
+      <c r="O9" s="3">
         <v>-1.42259</v>
       </c>
       <c r="P9" s="11"/>
@@ -3653,31 +3644,31 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" style="17" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="21" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="21" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="20" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="20" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="4" max="4" style="19" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="5" max="5" style="17" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="21" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="21" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="20" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="20" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="8" max="8" style="19" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="9" max="9" style="17" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="21" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="21" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="20" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="20" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="12" max="12" style="19" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="13" max="13" style="17" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="14" max="14" style="21" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="15" max="15" style="21" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="14" max="14" style="20" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="15" max="15" style="20" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="16" max="16" style="19" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="17" max="17" style="17" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="18" max="18" style="21" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="19" max="19" style="21" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="18" max="18" style="20" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="19" max="19" style="20" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="20" max="20" style="19" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="21" max="21" style="17" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="22" max="22" style="21" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="23" max="23" style="21" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="22" max="22" style="20" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="23" max="23" style="20" width="13.576428571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="15">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -3704,7 +3695,7 @@
       <c r="V1" s="3"/>
       <c r="W1" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
       <c r="A2" s="5" t="s">
         <v>1</v>
       </c>
@@ -5207,28 +5198,28 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" style="17" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="21" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="21" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="20" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="20" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="4" max="4" style="19" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="5" max="5" style="17" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="21" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="21" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="20" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="20" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="8" max="8" style="19" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="9" max="9" style="17" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="21" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="21" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="20" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="20" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="12" max="12" style="19" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="13" max="13" style="17" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="14" max="14" style="21" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="15" max="15" style="21" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="14" max="14" style="20" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="15" max="15" style="20" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="16" max="16" style="19" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="17" max="17" style="17" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="18" max="18" style="21" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="19" max="19" style="21" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="18" max="18" style="20" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="19" max="19" style="20" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="20" max="20" style="19" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="21" max="21" style="17" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="22" max="22" style="21" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="23" max="23" style="21" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="22" max="22" style="20" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="23" max="23" style="20" width="13.576428571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
@@ -6735,7 +6726,7 @@
       <c r="N26" s="14">
         <v>9.1516</v>
       </c>
-      <c r="O26" s="20">
+      <c r="O26" s="3">
         <v>-0.771998</v>
       </c>
       <c r="P26" s="11"/>
@@ -6769,1270 +6760,1231 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:AD26"/>
+  <dimension ref="A1:AC26"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="16" width="3.005" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="17" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="17" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="18" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="3" max="3" style="18" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="4" max="4" style="18" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="18" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="19" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="17" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="19" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="17" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="18" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="8" max="8" style="18" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="9" max="9" style="18" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="18" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="19" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="12" max="12" style="17" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="19" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="17" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="18" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="13" max="13" style="18" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="14" max="14" style="18" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="15" max="15" style="18" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="16" max="16" style="19" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="17" max="17" style="17" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="15" max="15" style="19" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="16" max="16" style="17" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="17" max="17" style="18" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="18" max="18" style="18" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="19" max="19" style="18" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="20" max="20" style="18" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="21" max="21" style="19" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="22" max="22" style="17" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="20" max="20" style="19" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="21" max="21" style="17" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="22" max="22" style="18" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="23" max="23" style="18" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="24" max="24" style="18" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="25" max="25" style="18" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="26" max="26" style="19" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="27" max="27" style="17" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="25" max="25" style="19" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="26" max="26" style="17" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="27" max="27" style="18" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="28" max="28" style="18" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="29" max="29" style="18" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="30" max="30" style="18" width="13.576428571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="15">
-      <c r="A1" s="1"/>
-      <c r="B1" s="2" t="s">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
+      <c r="B1" s="3"/>
       <c r="C1" s="3"/>
       <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="4"/>
-      <c r="G1" s="2"/>
+      <c r="E1" s="4"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="3"/>
       <c r="H1" s="3"/>
       <c r="I1" s="3"/>
-      <c r="J1" s="3"/>
-      <c r="K1" s="4"/>
-      <c r="L1" s="2"/>
+      <c r="J1" s="4"/>
+      <c r="K1" s="2"/>
+      <c r="L1" s="3"/>
       <c r="M1" s="3"/>
       <c r="N1" s="3"/>
-      <c r="O1" s="3"/>
-      <c r="P1" s="4"/>
-      <c r="Q1" s="2"/>
+      <c r="O1" s="4"/>
+      <c r="P1" s="2"/>
+      <c r="Q1" s="3"/>
       <c r="R1" s="3"/>
       <c r="S1" s="3"/>
-      <c r="T1" s="3"/>
-      <c r="U1" s="4"/>
-      <c r="V1" s="2"/>
+      <c r="T1" s="4"/>
+      <c r="U1" s="2"/>
+      <c r="V1" s="3"/>
       <c r="W1" s="3"/>
       <c r="X1" s="3"/>
-      <c r="Y1" s="3"/>
-      <c r="Z1" s="4"/>
-      <c r="AA1" s="2"/>
+      <c r="Y1" s="4"/>
+      <c r="Z1" s="2"/>
+      <c r="AA1" s="3"/>
       <c r="AB1" s="3"/>
       <c r="AC1" s="3"/>
-      <c r="AD1" s="3"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
-      <c r="A2" s="1"/>
-      <c r="B2" s="5" t="s">
+    </row>
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
+      <c r="A2" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="6"/>
-      <c r="D2" s="6" t="s">
+      <c r="B2" s="6"/>
+      <c r="C2" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="6"/>
-      <c r="F2" s="4"/>
-      <c r="G2" s="5" t="s">
+      <c r="D2" s="6"/>
+      <c r="E2" s="4"/>
+      <c r="F2" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="H2" s="6"/>
-      <c r="I2" s="6" t="s">
+      <c r="G2" s="6"/>
+      <c r="H2" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="J2" s="6"/>
-      <c r="K2" s="4"/>
-      <c r="L2" s="5" t="s">
+      <c r="I2" s="6"/>
+      <c r="J2" s="4"/>
+      <c r="K2" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="M2" s="6"/>
-      <c r="N2" s="6" t="s">
+      <c r="L2" s="6"/>
+      <c r="M2" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="O2" s="6"/>
-      <c r="P2" s="4"/>
-      <c r="Q2" s="5" t="s">
+      <c r="N2" s="6"/>
+      <c r="O2" s="4"/>
+      <c r="P2" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="R2" s="6"/>
-      <c r="S2" s="6" t="s">
+      <c r="Q2" s="6"/>
+      <c r="R2" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="T2" s="6"/>
-      <c r="U2" s="4"/>
-      <c r="V2" s="5" t="s">
+      <c r="S2" s="6"/>
+      <c r="T2" s="4"/>
+      <c r="U2" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="W2" s="6"/>
-      <c r="X2" s="6" t="s">
+      <c r="V2" s="6"/>
+      <c r="W2" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="Y2" s="6"/>
-      <c r="Z2" s="4"/>
-      <c r="AA2" s="5" t="s">
+      <c r="X2" s="6"/>
+      <c r="Y2" s="4"/>
+      <c r="Z2" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="AB2" s="6"/>
-      <c r="AC2" s="6" t="s">
+      <c r="AA2" s="6"/>
+      <c r="AB2" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="AD2" s="6"/>
+      <c r="AC2" s="6"/>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
-      <c r="A3" s="1"/>
-      <c r="B3" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="C3" s="8"/>
-      <c r="D3" s="9">
+      <c r="A3" s="7"/>
+      <c r="B3" s="8"/>
+      <c r="C3" s="9">
         <v>11026</v>
       </c>
-      <c r="E3" s="10"/>
-      <c r="F3" s="11"/>
-      <c r="G3" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="H3" s="8"/>
-      <c r="I3" s="9">
+      <c r="D3" s="10"/>
+      <c r="E3" s="11"/>
+      <c r="F3" s="7"/>
+      <c r="G3" s="8"/>
+      <c r="H3" s="9">
         <v>13917</v>
       </c>
-      <c r="J3" s="10"/>
-      <c r="K3" s="11"/>
-      <c r="L3" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="M3" s="8"/>
-      <c r="N3" s="9">
+      <c r="I3" s="10"/>
+      <c r="J3" s="11"/>
+      <c r="K3" s="7"/>
+      <c r="L3" s="8"/>
+      <c r="M3" s="9">
         <v>9053</v>
       </c>
-      <c r="O3" s="10"/>
-      <c r="P3" s="11"/>
-      <c r="Q3" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="R3" s="8"/>
-      <c r="S3" s="9">
+      <c r="N3" s="10"/>
+      <c r="O3" s="11"/>
+      <c r="P3" s="7"/>
+      <c r="Q3" s="8"/>
+      <c r="R3" s="9">
         <v>27976</v>
       </c>
-      <c r="T3" s="10"/>
-      <c r="U3" s="11"/>
-      <c r="V3" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="W3" s="8"/>
-      <c r="X3" s="9">
+      <c r="S3" s="10"/>
+      <c r="T3" s="11"/>
+      <c r="U3" s="7"/>
+      <c r="V3" s="8"/>
+      <c r="W3" s="9">
         <v>25638</v>
       </c>
-      <c r="Y3" s="10"/>
-      <c r="Z3" s="11"/>
-      <c r="AA3" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="AB3" s="8"/>
-      <c r="AC3" s="9">
+      <c r="X3" s="10"/>
+      <c r="Y3" s="11"/>
+      <c r="Z3" s="7"/>
+      <c r="AA3" s="8"/>
+      <c r="AB3" s="9">
         <v>31579</v>
       </c>
-      <c r="AD3" s="10"/>
+      <c r="AC3" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
-      <c r="A4" s="1"/>
-      <c r="B4" s="12" t="s">
+      <c r="A4" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="13">
+      <c r="B4" s="13">
         <v>0.665977</v>
       </c>
+      <c r="C4" s="14">
+        <v>436.25</v>
+      </c>
       <c r="D4" s="14">
-        <v>436.25</v>
-      </c>
-      <c r="E4" s="14">
         <v>-694.134</v>
       </c>
-      <c r="F4" s="11"/>
-      <c r="G4" s="12" t="s">
+      <c r="E4" s="11"/>
+      <c r="F4" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="H4" s="13">
+      <c r="G4" s="13">
         <v>3.80731</v>
       </c>
+      <c r="H4" s="14">
+        <v>446.408</v>
+      </c>
       <c r="I4" s="14">
-        <v>446.408</v>
-      </c>
-      <c r="J4" s="14">
         <v>-693.016</v>
       </c>
-      <c r="K4" s="11"/>
-      <c r="L4" s="12" t="s">
+      <c r="J4" s="11"/>
+      <c r="K4" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="M4" s="13">
+      <c r="L4" s="13">
         <v>-5.06056</v>
       </c>
+      <c r="M4" s="14">
+        <v>445.116</v>
+      </c>
       <c r="N4" s="14">
-        <v>445.116</v>
-      </c>
-      <c r="O4" s="14">
         <v>-691.777</v>
       </c>
-      <c r="P4" s="11"/>
-      <c r="Q4" s="12" t="s">
+      <c r="O4" s="11"/>
+      <c r="P4" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="R4" s="13">
+      <c r="Q4" s="13">
         <v>-0.409241</v>
       </c>
+      <c r="R4" s="14">
+        <v>435.893</v>
+      </c>
       <c r="S4" s="14">
-        <v>435.893</v>
-      </c>
-      <c r="T4" s="14">
         <v>-700.587</v>
       </c>
-      <c r="U4" s="11"/>
-      <c r="V4" s="12" t="s">
+      <c r="T4" s="11"/>
+      <c r="U4" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="W4" s="13">
+      <c r="V4" s="13">
         <v>-7.73474</v>
       </c>
+      <c r="W4" s="14">
+        <v>443.012</v>
+      </c>
       <c r="X4" s="14">
-        <v>443.012</v>
-      </c>
-      <c r="Y4" s="14">
         <v>-696.511</v>
       </c>
-      <c r="Z4" s="11"/>
-      <c r="AA4" s="12" t="s">
+      <c r="Y4" s="11"/>
+      <c r="Z4" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="AB4" s="13">
+      <c r="AA4" s="13">
         <v>8.37844</v>
       </c>
+      <c r="AB4" s="14">
+        <v>443.66</v>
+      </c>
       <c r="AC4" s="14">
-        <v>443.66</v>
-      </c>
-      <c r="AD4" s="14">
         <v>-697.608</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
-      <c r="A5" s="1"/>
-      <c r="B5" s="15" t="s">
+      <c r="A5" s="15" t="s">
         <v>11</v>
       </c>
+      <c r="B5" s="10" t="s">
+        <v>12</v>
+      </c>
       <c r="C5" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="E5" s="11"/>
+      <c r="F5" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="G5" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="D5" s="10" t="s">
+      <c r="H5" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="E5" s="10" t="s">
+      <c r="I5" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="F5" s="11"/>
-      <c r="G5" s="15" t="s">
+      <c r="J5" s="11"/>
+      <c r="K5" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="H5" s="10" t="s">
+      <c r="L5" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="I5" s="10" t="s">
+      <c r="M5" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="J5" s="10" t="s">
+      <c r="N5" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="K5" s="11"/>
-      <c r="L5" s="15" t="s">
+      <c r="O5" s="11"/>
+      <c r="P5" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="M5" s="10" t="s">
+      <c r="Q5" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="N5" s="10" t="s">
+      <c r="R5" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="O5" s="10" t="s">
+      <c r="S5" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="P5" s="11"/>
-      <c r="Q5" s="15" t="s">
+      <c r="T5" s="11"/>
+      <c r="U5" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="R5" s="10" t="s">
+      <c r="V5" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="S5" s="10" t="s">
+      <c r="W5" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="T5" s="10" t="s">
+      <c r="X5" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="U5" s="11"/>
-      <c r="V5" s="15" t="s">
+      <c r="Y5" s="11"/>
+      <c r="Z5" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="W5" s="10" t="s">
+      <c r="AA5" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="X5" s="10" t="s">
+      <c r="AB5" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="Y5" s="10" t="s">
+      <c r="AC5" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="Z5" s="11"/>
-      <c r="AA5" s="15" t="s">
-        <v>11</v>
-      </c>
-      <c r="AB5" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="AC5" s="10" t="s">
-        <v>13</v>
-      </c>
-      <c r="AD5" s="10" t="s">
-        <v>14</v>
-      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
-      <c r="A6" s="1"/>
-      <c r="B6" s="9">
+      <c r="A6" s="9">
         <v>0</v>
       </c>
+      <c r="B6" s="10"/>
       <c r="C6" s="10"/>
       <c r="D6" s="10"/>
-      <c r="E6" s="10"/>
-      <c r="F6" s="11"/>
-      <c r="G6" s="9">
+      <c r="E6" s="11"/>
+      <c r="F6" s="9">
         <v>0</v>
       </c>
+      <c r="G6" s="10"/>
       <c r="H6" s="10"/>
       <c r="I6" s="10"/>
-      <c r="J6" s="10"/>
-      <c r="K6" s="11"/>
-      <c r="L6" s="9">
+      <c r="J6" s="11"/>
+      <c r="K6" s="9">
         <v>0</v>
       </c>
+      <c r="L6" s="10"/>
       <c r="M6" s="10"/>
       <c r="N6" s="10"/>
-      <c r="O6" s="10"/>
-      <c r="P6" s="11"/>
-      <c r="Q6" s="9">
+      <c r="O6" s="11"/>
+      <c r="P6" s="9">
         <v>0</v>
       </c>
+      <c r="Q6" s="10"/>
       <c r="R6" s="10"/>
       <c r="S6" s="10"/>
-      <c r="T6" s="10"/>
-      <c r="U6" s="11"/>
-      <c r="V6" s="9">
+      <c r="T6" s="11"/>
+      <c r="U6" s="9">
         <v>0</v>
       </c>
+      <c r="V6" s="10"/>
       <c r="W6" s="10"/>
       <c r="X6" s="10"/>
-      <c r="Y6" s="10"/>
-      <c r="Z6" s="11"/>
-      <c r="AA6" s="9">
+      <c r="Y6" s="11"/>
+      <c r="Z6" s="9">
         <v>0</v>
       </c>
+      <c r="AA6" s="10"/>
       <c r="AB6" s="10"/>
       <c r="AC6" s="10"/>
-      <c r="AD6" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
-      <c r="A7" s="1"/>
-      <c r="B7" s="14">
+      <c r="A7" s="14">
         <v>0.05</v>
       </c>
+      <c r="B7" s="10"/>
       <c r="C7" s="10"/>
       <c r="D7" s="10"/>
-      <c r="E7" s="10"/>
-      <c r="F7" s="11"/>
-      <c r="G7" s="14">
+      <c r="E7" s="11"/>
+      <c r="F7" s="14">
         <v>0.05</v>
       </c>
+      <c r="G7" s="10"/>
       <c r="H7" s="10"/>
       <c r="I7" s="10"/>
-      <c r="J7" s="10"/>
-      <c r="K7" s="11"/>
-      <c r="L7" s="14">
+      <c r="J7" s="11"/>
+      <c r="K7" s="14">
         <v>0.05</v>
       </c>
+      <c r="L7" s="10"/>
       <c r="M7" s="10"/>
       <c r="N7" s="10"/>
-      <c r="O7" s="10"/>
-      <c r="P7" s="11"/>
-      <c r="Q7" s="14">
+      <c r="O7" s="11"/>
+      <c r="P7" s="14">
         <v>0.05</v>
       </c>
+      <c r="Q7" s="10"/>
       <c r="R7" s="10"/>
       <c r="S7" s="10"/>
-      <c r="T7" s="10"/>
-      <c r="U7" s="11"/>
-      <c r="V7" s="14">
+      <c r="T7" s="11"/>
+      <c r="U7" s="14">
         <v>0.05</v>
       </c>
+      <c r="V7" s="10"/>
       <c r="W7" s="10"/>
       <c r="X7" s="10"/>
-      <c r="Y7" s="10"/>
-      <c r="Z7" s="11"/>
-      <c r="AA7" s="14">
+      <c r="Y7" s="11"/>
+      <c r="Z7" s="14">
         <v>0.05</v>
       </c>
+      <c r="AA7" s="10"/>
       <c r="AB7" s="10"/>
       <c r="AC7" s="10"/>
-      <c r="AD7" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
-      <c r="A8" s="1"/>
-      <c r="B8" s="14">
+      <c r="A8" s="14">
         <v>0.1</v>
       </c>
+      <c r="B8" s="10"/>
       <c r="C8" s="10"/>
       <c r="D8" s="10"/>
-      <c r="E8" s="10"/>
-      <c r="F8" s="11"/>
-      <c r="G8" s="14">
+      <c r="E8" s="11"/>
+      <c r="F8" s="14">
         <v>0.1</v>
       </c>
+      <c r="G8" s="10"/>
       <c r="H8" s="10"/>
       <c r="I8" s="10"/>
-      <c r="J8" s="10"/>
-      <c r="K8" s="11"/>
-      <c r="L8" s="14">
+      <c r="J8" s="11"/>
+      <c r="K8" s="14">
         <v>0.1</v>
       </c>
+      <c r="L8" s="10"/>
       <c r="M8" s="10"/>
       <c r="N8" s="10"/>
-      <c r="O8" s="10"/>
-      <c r="P8" s="11"/>
-      <c r="Q8" s="14">
+      <c r="O8" s="11"/>
+      <c r="P8" s="14">
         <v>0.1</v>
       </c>
+      <c r="Q8" s="10"/>
       <c r="R8" s="10"/>
       <c r="S8" s="10"/>
-      <c r="T8" s="10"/>
-      <c r="U8" s="11"/>
-      <c r="V8" s="14">
+      <c r="T8" s="11"/>
+      <c r="U8" s="14">
         <v>0.1</v>
       </c>
+      <c r="V8" s="10"/>
       <c r="W8" s="10"/>
       <c r="X8" s="10"/>
-      <c r="Y8" s="10"/>
-      <c r="Z8" s="11"/>
-      <c r="AA8" s="14">
+      <c r="Y8" s="11"/>
+      <c r="Z8" s="14">
         <v>0.1</v>
       </c>
+      <c r="AA8" s="10"/>
       <c r="AB8" s="10"/>
       <c r="AC8" s="10"/>
-      <c r="AD8" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
-      <c r="A9" s="1"/>
-      <c r="B9" s="14">
+      <c r="A9" s="14">
         <v>0.15</v>
       </c>
+      <c r="B9" s="10"/>
       <c r="C9" s="10"/>
       <c r="D9" s="10"/>
-      <c r="E9" s="10"/>
-      <c r="F9" s="11"/>
-      <c r="G9" s="14">
+      <c r="E9" s="11"/>
+      <c r="F9" s="14">
         <v>0.15</v>
       </c>
+      <c r="G9" s="10"/>
       <c r="H9" s="10"/>
       <c r="I9" s="10"/>
-      <c r="J9" s="10"/>
-      <c r="K9" s="11"/>
-      <c r="L9" s="14">
+      <c r="J9" s="11"/>
+      <c r="K9" s="14">
         <v>0.15</v>
       </c>
+      <c r="L9" s="10"/>
       <c r="M9" s="10"/>
       <c r="N9" s="10"/>
-      <c r="O9" s="10"/>
-      <c r="P9" s="11"/>
-      <c r="Q9" s="14">
+      <c r="O9" s="11"/>
+      <c r="P9" s="14">
         <v>0.15</v>
       </c>
+      <c r="Q9" s="10"/>
       <c r="R9" s="10"/>
       <c r="S9" s="10"/>
-      <c r="T9" s="10"/>
-      <c r="U9" s="11"/>
-      <c r="V9" s="14">
+      <c r="T9" s="11"/>
+      <c r="U9" s="14">
         <v>0.15</v>
       </c>
+      <c r="V9" s="10"/>
       <c r="W9" s="10"/>
       <c r="X9" s="10"/>
-      <c r="Y9" s="10"/>
-      <c r="Z9" s="11"/>
-      <c r="AA9" s="14">
+      <c r="Y9" s="11"/>
+      <c r="Z9" s="14">
         <v>0.15</v>
       </c>
+      <c r="AA9" s="10"/>
       <c r="AB9" s="10"/>
       <c r="AC9" s="10"/>
-      <c r="AD9" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
-      <c r="A10" s="1"/>
-      <c r="B10" s="14">
+      <c r="A10" s="14">
         <v>0.2</v>
       </c>
+      <c r="B10" s="10"/>
       <c r="C10" s="10"/>
       <c r="D10" s="10"/>
-      <c r="E10" s="10"/>
-      <c r="F10" s="11"/>
-      <c r="G10" s="14">
+      <c r="E10" s="11"/>
+      <c r="F10" s="14">
         <v>0.2</v>
       </c>
+      <c r="G10" s="10"/>
       <c r="H10" s="10"/>
       <c r="I10" s="10"/>
-      <c r="J10" s="10"/>
-      <c r="K10" s="11"/>
-      <c r="L10" s="14">
+      <c r="J10" s="11"/>
+      <c r="K10" s="14">
         <v>0.2</v>
       </c>
+      <c r="L10" s="10"/>
       <c r="M10" s="10"/>
       <c r="N10" s="10"/>
-      <c r="O10" s="10"/>
-      <c r="P10" s="11"/>
-      <c r="Q10" s="14">
+      <c r="O10" s="11"/>
+      <c r="P10" s="14">
         <v>0.2</v>
       </c>
+      <c r="Q10" s="10"/>
       <c r="R10" s="10"/>
       <c r="S10" s="10"/>
-      <c r="T10" s="10"/>
-      <c r="U10" s="11"/>
-      <c r="V10" s="14">
+      <c r="T10" s="11"/>
+      <c r="U10" s="14">
         <v>0.2</v>
       </c>
+      <c r="V10" s="10"/>
       <c r="W10" s="10"/>
       <c r="X10" s="10"/>
-      <c r="Y10" s="10"/>
-      <c r="Z10" s="11"/>
-      <c r="AA10" s="14">
+      <c r="Y10" s="11"/>
+      <c r="Z10" s="14">
         <v>0.2</v>
       </c>
+      <c r="AA10" s="10"/>
       <c r="AB10" s="10"/>
       <c r="AC10" s="10"/>
-      <c r="AD10" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
-      <c r="A11" s="1"/>
-      <c r="B11" s="14">
+      <c r="A11" s="14">
         <v>0.25</v>
       </c>
+      <c r="B11" s="10"/>
       <c r="C11" s="10"/>
       <c r="D11" s="10"/>
-      <c r="E11" s="10"/>
-      <c r="F11" s="11"/>
-      <c r="G11" s="14">
+      <c r="E11" s="11"/>
+      <c r="F11" s="14">
         <v>0.25</v>
       </c>
+      <c r="G11" s="10"/>
       <c r="H11" s="10"/>
       <c r="I11" s="10"/>
-      <c r="J11" s="10"/>
-      <c r="K11" s="11"/>
-      <c r="L11" s="14">
+      <c r="J11" s="11"/>
+      <c r="K11" s="14">
         <v>0.25</v>
       </c>
+      <c r="L11" s="10"/>
       <c r="M11" s="10"/>
       <c r="N11" s="10"/>
-      <c r="O11" s="10"/>
-      <c r="P11" s="11"/>
-      <c r="Q11" s="14">
+      <c r="O11" s="11"/>
+      <c r="P11" s="14">
         <v>0.25</v>
       </c>
+      <c r="Q11" s="10"/>
       <c r="R11" s="10"/>
       <c r="S11" s="10"/>
-      <c r="T11" s="10"/>
-      <c r="U11" s="11"/>
-      <c r="V11" s="14">
+      <c r="T11" s="11"/>
+      <c r="U11" s="14">
         <v>0.25</v>
       </c>
+      <c r="V11" s="10"/>
       <c r="W11" s="10"/>
       <c r="X11" s="10"/>
-      <c r="Y11" s="10"/>
-      <c r="Z11" s="11"/>
-      <c r="AA11" s="14">
+      <c r="Y11" s="11"/>
+      <c r="Z11" s="14">
         <v>0.25</v>
       </c>
+      <c r="AA11" s="10"/>
       <c r="AB11" s="10"/>
       <c r="AC11" s="10"/>
-      <c r="AD11" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75">
-      <c r="A12" s="1"/>
-      <c r="B12" s="14">
+      <c r="A12" s="14">
         <v>0.30198</v>
       </c>
+      <c r="B12" s="10"/>
       <c r="C12" s="10"/>
       <c r="D12" s="10"/>
-      <c r="E12" s="10"/>
-      <c r="F12" s="11"/>
-      <c r="G12" s="14">
+      <c r="E12" s="11"/>
+      <c r="F12" s="14">
         <v>0.30198</v>
       </c>
+      <c r="G12" s="10"/>
       <c r="H12" s="10"/>
       <c r="I12" s="10"/>
-      <c r="J12" s="10"/>
-      <c r="K12" s="11"/>
-      <c r="L12" s="14">
+      <c r="J12" s="11"/>
+      <c r="K12" s="14">
         <v>0.30198</v>
       </c>
+      <c r="L12" s="10"/>
       <c r="M12" s="10"/>
       <c r="N12" s="10"/>
-      <c r="O12" s="10"/>
-      <c r="P12" s="11"/>
-      <c r="Q12" s="14">
+      <c r="O12" s="11"/>
+      <c r="P12" s="14">
         <v>0.30198</v>
       </c>
+      <c r="Q12" s="10"/>
       <c r="R12" s="10"/>
       <c r="S12" s="10"/>
-      <c r="T12" s="10"/>
-      <c r="U12" s="11"/>
-      <c r="V12" s="14">
+      <c r="T12" s="11"/>
+      <c r="U12" s="14">
         <v>0.30198</v>
       </c>
+      <c r="V12" s="10"/>
       <c r="W12" s="10"/>
       <c r="X12" s="10"/>
-      <c r="Y12" s="10"/>
-      <c r="Z12" s="11"/>
-      <c r="AA12" s="14">
+      <c r="Y12" s="11"/>
+      <c r="Z12" s="14">
         <v>0.30198</v>
       </c>
+      <c r="AA12" s="10"/>
       <c r="AB12" s="10"/>
       <c r="AC12" s="10"/>
-      <c r="AD12" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75">
-      <c r="A13" s="1"/>
-      <c r="B13" s="14">
+      <c r="A13" s="14">
         <v>0.35365</v>
       </c>
+      <c r="B13" s="10"/>
       <c r="C13" s="10"/>
       <c r="D13" s="10"/>
-      <c r="E13" s="10"/>
-      <c r="F13" s="11"/>
-      <c r="G13" s="14">
+      <c r="E13" s="11"/>
+      <c r="F13" s="14">
         <v>0.35365</v>
       </c>
+      <c r="G13" s="10"/>
       <c r="H13" s="10"/>
       <c r="I13" s="10"/>
-      <c r="J13" s="10"/>
-      <c r="K13" s="11"/>
-      <c r="L13" s="14">
+      <c r="J13" s="11"/>
+      <c r="K13" s="14">
         <v>0.35365</v>
       </c>
+      <c r="L13" s="10"/>
       <c r="M13" s="10"/>
       <c r="N13" s="10"/>
-      <c r="O13" s="10"/>
-      <c r="P13" s="11"/>
-      <c r="Q13" s="14">
+      <c r="O13" s="11"/>
+      <c r="P13" s="14">
         <v>0.35365</v>
       </c>
+      <c r="Q13" s="10"/>
       <c r="R13" s="10"/>
       <c r="S13" s="10"/>
-      <c r="T13" s="10"/>
-      <c r="U13" s="11"/>
-      <c r="V13" s="14">
+      <c r="T13" s="11"/>
+      <c r="U13" s="14">
         <v>0.35365</v>
       </c>
+      <c r="V13" s="10"/>
       <c r="W13" s="10"/>
       <c r="X13" s="10"/>
-      <c r="Y13" s="10"/>
-      <c r="Z13" s="11"/>
-      <c r="AA13" s="14">
+      <c r="Y13" s="11"/>
+      <c r="Z13" s="14">
         <v>0.35365</v>
       </c>
+      <c r="AA13" s="10"/>
       <c r="AB13" s="10"/>
       <c r="AC13" s="10"/>
-      <c r="AD13" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18.75">
-      <c r="A14" s="1"/>
-      <c r="B14" s="14">
+      <c r="A14" s="14">
         <v>0.40358</v>
       </c>
+      <c r="B14" s="10"/>
       <c r="C14" s="10"/>
       <c r="D14" s="10"/>
-      <c r="E14" s="10"/>
-      <c r="F14" s="11"/>
-      <c r="G14" s="14">
+      <c r="E14" s="11"/>
+      <c r="F14" s="14">
         <v>0.40358</v>
       </c>
+      <c r="G14" s="10"/>
       <c r="H14" s="10"/>
       <c r="I14" s="10"/>
-      <c r="J14" s="10"/>
-      <c r="K14" s="11"/>
-      <c r="L14" s="14">
+      <c r="J14" s="11"/>
+      <c r="K14" s="14">
         <v>0.40358</v>
       </c>
+      <c r="L14" s="10"/>
       <c r="M14" s="10"/>
       <c r="N14" s="10"/>
-      <c r="O14" s="10"/>
-      <c r="P14" s="11"/>
-      <c r="Q14" s="14">
+      <c r="O14" s="11"/>
+      <c r="P14" s="14">
         <v>0.40358</v>
       </c>
+      <c r="Q14" s="10"/>
       <c r="R14" s="10"/>
       <c r="S14" s="10"/>
-      <c r="T14" s="10"/>
-      <c r="U14" s="11"/>
-      <c r="V14" s="14">
+      <c r="T14" s="11"/>
+      <c r="U14" s="14">
         <v>0.40358</v>
       </c>
+      <c r="V14" s="10"/>
       <c r="W14" s="10"/>
       <c r="X14" s="10"/>
-      <c r="Y14" s="10"/>
-      <c r="Z14" s="11"/>
-      <c r="AA14" s="14">
+      <c r="Y14" s="11"/>
+      <c r="Z14" s="14">
         <v>0.40358</v>
       </c>
+      <c r="AA14" s="10"/>
       <c r="AB14" s="10"/>
       <c r="AC14" s="10"/>
-      <c r="AD14" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18.75">
-      <c r="A15" s="1"/>
-      <c r="B15" s="14">
+      <c r="A15" s="14">
         <v>0.45421</v>
       </c>
+      <c r="B15" s="10"/>
       <c r="C15" s="10"/>
       <c r="D15" s="10"/>
-      <c r="E15" s="10"/>
-      <c r="F15" s="11"/>
-      <c r="G15" s="14">
+      <c r="E15" s="11"/>
+      <c r="F15" s="14">
         <v>0.45421</v>
       </c>
+      <c r="G15" s="10"/>
       <c r="H15" s="10"/>
       <c r="I15" s="10"/>
-      <c r="J15" s="10"/>
-      <c r="K15" s="11"/>
-      <c r="L15" s="14">
+      <c r="J15" s="11"/>
+      <c r="K15" s="14">
         <v>0.45421</v>
       </c>
+      <c r="L15" s="10"/>
       <c r="M15" s="10"/>
       <c r="N15" s="10"/>
-      <c r="O15" s="10"/>
-      <c r="P15" s="11"/>
-      <c r="Q15" s="14">
+      <c r="O15" s="11"/>
+      <c r="P15" s="14">
         <v>0.45421</v>
       </c>
+      <c r="Q15" s="10"/>
       <c r="R15" s="10"/>
       <c r="S15" s="10"/>
-      <c r="T15" s="10"/>
-      <c r="U15" s="11"/>
-      <c r="V15" s="14">
+      <c r="T15" s="11"/>
+      <c r="U15" s="14">
         <v>0.45421</v>
       </c>
+      <c r="V15" s="10"/>
       <c r="W15" s="10"/>
       <c r="X15" s="10"/>
-      <c r="Y15" s="10"/>
-      <c r="Z15" s="11"/>
-      <c r="AA15" s="14">
+      <c r="Y15" s="11"/>
+      <c r="Z15" s="14">
         <v>0.45421</v>
       </c>
+      <c r="AA15" s="10"/>
       <c r="AB15" s="10"/>
       <c r="AC15" s="10"/>
-      <c r="AD15" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18.75">
-      <c r="A16" s="1"/>
-      <c r="B16" s="14">
+      <c r="A16" s="14">
         <v>0.50322</v>
       </c>
+      <c r="B16" s="10"/>
       <c r="C16" s="10"/>
       <c r="D16" s="10"/>
-      <c r="E16" s="10"/>
-      <c r="F16" s="11"/>
-      <c r="G16" s="14">
+      <c r="E16" s="11"/>
+      <c r="F16" s="14">
         <v>0.50322</v>
       </c>
+      <c r="G16" s="10"/>
       <c r="H16" s="10"/>
       <c r="I16" s="10"/>
-      <c r="J16" s="10"/>
-      <c r="K16" s="11"/>
-      <c r="L16" s="14">
+      <c r="J16" s="11"/>
+      <c r="K16" s="14">
         <v>0.50322</v>
       </c>
+      <c r="L16" s="10"/>
       <c r="M16" s="10"/>
       <c r="N16" s="10"/>
-      <c r="O16" s="10"/>
-      <c r="P16" s="11"/>
-      <c r="Q16" s="14">
+      <c r="O16" s="11"/>
+      <c r="P16" s="14">
         <v>0.50322</v>
       </c>
+      <c r="Q16" s="10"/>
       <c r="R16" s="10"/>
       <c r="S16" s="10"/>
-      <c r="T16" s="10"/>
-      <c r="U16" s="11"/>
-      <c r="V16" s="14">
+      <c r="T16" s="11"/>
+      <c r="U16" s="14">
         <v>0.50322</v>
       </c>
+      <c r="V16" s="10"/>
       <c r="W16" s="10"/>
       <c r="X16" s="10"/>
-      <c r="Y16" s="10"/>
-      <c r="Z16" s="11"/>
-      <c r="AA16" s="14">
+      <c r="Y16" s="11"/>
+      <c r="Z16" s="14">
         <v>0.50322</v>
       </c>
+      <c r="AA16" s="10"/>
       <c r="AB16" s="10"/>
       <c r="AC16" s="10"/>
-      <c r="AD16" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18.75">
-      <c r="A17" s="1"/>
-      <c r="B17" s="14">
+      <c r="A17" s="14">
         <v>0.55384</v>
       </c>
+      <c r="B17" s="10"/>
       <c r="C17" s="10"/>
       <c r="D17" s="10"/>
-      <c r="E17" s="10"/>
-      <c r="F17" s="11"/>
-      <c r="G17" s="14">
+      <c r="E17" s="11"/>
+      <c r="F17" s="14">
         <v>0.55384</v>
       </c>
+      <c r="G17" s="10"/>
       <c r="H17" s="10"/>
       <c r="I17" s="10"/>
-      <c r="J17" s="10"/>
-      <c r="K17" s="11"/>
-      <c r="L17" s="14">
+      <c r="J17" s="11"/>
+      <c r="K17" s="14">
         <v>0.55384</v>
       </c>
+      <c r="L17" s="10"/>
       <c r="M17" s="10"/>
       <c r="N17" s="10"/>
-      <c r="O17" s="10"/>
-      <c r="P17" s="11"/>
-      <c r="Q17" s="14">
+      <c r="O17" s="11"/>
+      <c r="P17" s="14">
         <v>0.55384</v>
       </c>
+      <c r="Q17" s="10"/>
       <c r="R17" s="10"/>
       <c r="S17" s="10"/>
-      <c r="T17" s="10"/>
-      <c r="U17" s="11"/>
-      <c r="V17" s="14">
+      <c r="T17" s="11"/>
+      <c r="U17" s="14">
         <v>0.55384</v>
       </c>
+      <c r="V17" s="10"/>
       <c r="W17" s="10"/>
       <c r="X17" s="10"/>
-      <c r="Y17" s="10"/>
-      <c r="Z17" s="11"/>
-      <c r="AA17" s="14">
+      <c r="Y17" s="11"/>
+      <c r="Z17" s="14">
         <v>0.55384</v>
       </c>
+      <c r="AA17" s="10"/>
       <c r="AB17" s="10"/>
       <c r="AC17" s="10"/>
-      <c r="AD17" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="18.75">
-      <c r="A18" s="1"/>
-      <c r="B18" s="14">
+      <c r="A18" s="14">
         <v>0.60384</v>
       </c>
+      <c r="B18" s="10"/>
       <c r="C18" s="10"/>
       <c r="D18" s="10"/>
-      <c r="E18" s="10"/>
-      <c r="F18" s="11"/>
-      <c r="G18" s="14">
+      <c r="E18" s="11"/>
+      <c r="F18" s="14">
         <v>0.60384</v>
       </c>
+      <c r="G18" s="10"/>
       <c r="H18" s="10"/>
       <c r="I18" s="10"/>
-      <c r="J18" s="10"/>
-      <c r="K18" s="11"/>
-      <c r="L18" s="14">
+      <c r="J18" s="11"/>
+      <c r="K18" s="14">
         <v>0.60384</v>
       </c>
+      <c r="L18" s="10"/>
       <c r="M18" s="10"/>
       <c r="N18" s="10"/>
-      <c r="O18" s="10"/>
-      <c r="P18" s="11"/>
-      <c r="Q18" s="14">
+      <c r="O18" s="11"/>
+      <c r="P18" s="14">
         <v>0.60384</v>
       </c>
+      <c r="Q18" s="10"/>
       <c r="R18" s="10"/>
       <c r="S18" s="10"/>
-      <c r="T18" s="10"/>
-      <c r="U18" s="11"/>
-      <c r="V18" s="14">
+      <c r="T18" s="11"/>
+      <c r="U18" s="14">
         <v>0.60384</v>
       </c>
+      <c r="V18" s="10"/>
       <c r="W18" s="10"/>
       <c r="X18" s="10"/>
-      <c r="Y18" s="10"/>
-      <c r="Z18" s="11"/>
-      <c r="AA18" s="14">
+      <c r="Y18" s="11"/>
+      <c r="Z18" s="14">
         <v>0.60384</v>
       </c>
+      <c r="AA18" s="10"/>
       <c r="AB18" s="10"/>
       <c r="AC18" s="10"/>
-      <c r="AD18" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="18.75">
-      <c r="A19" s="1"/>
-      <c r="B19" s="14">
+      <c r="A19" s="14">
         <v>0.65565</v>
       </c>
+      <c r="B19" s="10"/>
       <c r="C19" s="10"/>
       <c r="D19" s="10"/>
-      <c r="E19" s="10"/>
-      <c r="F19" s="11"/>
-      <c r="G19" s="14">
+      <c r="E19" s="11"/>
+      <c r="F19" s="14">
         <v>0.65565</v>
       </c>
+      <c r="G19" s="10"/>
       <c r="H19" s="10"/>
       <c r="I19" s="10"/>
-      <c r="J19" s="10"/>
-      <c r="K19" s="11"/>
-      <c r="L19" s="14">
+      <c r="J19" s="11"/>
+      <c r="K19" s="14">
         <v>0.65565</v>
       </c>
+      <c r="L19" s="10"/>
       <c r="M19" s="10"/>
       <c r="N19" s="10"/>
-      <c r="O19" s="10"/>
-      <c r="P19" s="11"/>
-      <c r="Q19" s="14">
+      <c r="O19" s="11"/>
+      <c r="P19" s="14">
         <v>0.65565</v>
       </c>
+      <c r="Q19" s="10"/>
       <c r="R19" s="10"/>
       <c r="S19" s="10"/>
-      <c r="T19" s="10"/>
-      <c r="U19" s="11"/>
-      <c r="V19" s="14">
+      <c r="T19" s="11"/>
+      <c r="U19" s="14">
         <v>0.65565</v>
       </c>
+      <c r="V19" s="10"/>
       <c r="W19" s="10"/>
       <c r="X19" s="10"/>
-      <c r="Y19" s="10"/>
-      <c r="Z19" s="11"/>
-      <c r="AA19" s="14">
+      <c r="Y19" s="11"/>
+      <c r="Z19" s="14">
         <v>0.65565</v>
       </c>
+      <c r="AA19" s="10"/>
       <c r="AB19" s="10"/>
       <c r="AC19" s="10"/>
-      <c r="AD19" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="18.75">
-      <c r="A20" s="1"/>
-      <c r="B20" s="14">
+      <c r="A20" s="14">
         <v>0.70225</v>
       </c>
+      <c r="B20" s="10"/>
       <c r="C20" s="10"/>
       <c r="D20" s="10"/>
-      <c r="E20" s="10"/>
-      <c r="F20" s="11"/>
-      <c r="G20" s="14">
+      <c r="E20" s="11"/>
+      <c r="F20" s="14">
         <v>0.70225</v>
       </c>
+      <c r="G20" s="10"/>
       <c r="H20" s="10"/>
       <c r="I20" s="10"/>
-      <c r="J20" s="10"/>
-      <c r="K20" s="11"/>
-      <c r="L20" s="14">
+      <c r="J20" s="11"/>
+      <c r="K20" s="14">
         <v>0.70225</v>
       </c>
+      <c r="L20" s="10"/>
       <c r="M20" s="10"/>
       <c r="N20" s="10"/>
-      <c r="O20" s="10"/>
-      <c r="P20" s="11"/>
-      <c r="Q20" s="14">
+      <c r="O20" s="11"/>
+      <c r="P20" s="14">
         <v>0.70225</v>
       </c>
+      <c r="Q20" s="10"/>
       <c r="R20" s="10"/>
       <c r="S20" s="10"/>
-      <c r="T20" s="10"/>
-      <c r="U20" s="11"/>
-      <c r="V20" s="14">
+      <c r="T20" s="11"/>
+      <c r="U20" s="14">
         <v>0.70225</v>
       </c>
+      <c r="V20" s="10"/>
       <c r="W20" s="10"/>
       <c r="X20" s="10"/>
-      <c r="Y20" s="10"/>
-      <c r="Z20" s="11"/>
-      <c r="AA20" s="14">
+      <c r="Y20" s="11"/>
+      <c r="Z20" s="14">
         <v>0.70225</v>
       </c>
+      <c r="AA20" s="10"/>
       <c r="AB20" s="10"/>
       <c r="AC20" s="10"/>
-      <c r="AD20" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="18.75">
-      <c r="A21" s="1"/>
-      <c r="B21" s="14">
+      <c r="A21" s="14">
         <v>0.75206</v>
       </c>
+      <c r="B21" s="10"/>
       <c r="C21" s="10"/>
       <c r="D21" s="10"/>
-      <c r="E21" s="10"/>
-      <c r="F21" s="11"/>
-      <c r="G21" s="14">
+      <c r="E21" s="11"/>
+      <c r="F21" s="14">
         <v>0.75206</v>
       </c>
+      <c r="G21" s="10"/>
       <c r="H21" s="10"/>
       <c r="I21" s="10"/>
-      <c r="J21" s="10"/>
-      <c r="K21" s="11"/>
-      <c r="L21" s="14">
+      <c r="J21" s="11"/>
+      <c r="K21" s="14">
         <v>0.75206</v>
       </c>
+      <c r="L21" s="10"/>
       <c r="M21" s="10"/>
       <c r="N21" s="10"/>
-      <c r="O21" s="10"/>
-      <c r="P21" s="11"/>
-      <c r="Q21" s="14">
+      <c r="O21" s="11"/>
+      <c r="P21" s="14">
         <v>0.75206</v>
       </c>
+      <c r="Q21" s="10"/>
       <c r="R21" s="10"/>
       <c r="S21" s="10"/>
-      <c r="T21" s="10"/>
-      <c r="U21" s="11"/>
-      <c r="V21" s="14">
+      <c r="T21" s="11"/>
+      <c r="U21" s="14">
         <v>0.75206</v>
       </c>
+      <c r="V21" s="10"/>
       <c r="W21" s="10"/>
       <c r="X21" s="10"/>
-      <c r="Y21" s="10"/>
-      <c r="Z21" s="11"/>
-      <c r="AA21" s="14">
+      <c r="Y21" s="11"/>
+      <c r="Z21" s="14">
         <v>0.75206</v>
       </c>
+      <c r="AA21" s="10"/>
       <c r="AB21" s="10"/>
       <c r="AC21" s="10"/>
-      <c r="AD21" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="18.75">
-      <c r="A22" s="1"/>
-      <c r="B22" s="14">
+      <c r="A22" s="14">
         <v>0.80139</v>
       </c>
+      <c r="B22" s="10"/>
       <c r="C22" s="10"/>
       <c r="D22" s="10"/>
-      <c r="E22" s="10"/>
-      <c r="F22" s="11"/>
-      <c r="G22" s="14">
+      <c r="E22" s="11"/>
+      <c r="F22" s="14">
         <v>0.80139</v>
       </c>
+      <c r="G22" s="10"/>
       <c r="H22" s="10"/>
       <c r="I22" s="10"/>
-      <c r="J22" s="10"/>
-      <c r="K22" s="11"/>
-      <c r="L22" s="14">
+      <c r="J22" s="11"/>
+      <c r="K22" s="14">
         <v>0.80139</v>
       </c>
+      <c r="L22" s="10"/>
       <c r="M22" s="10"/>
       <c r="N22" s="10"/>
-      <c r="O22" s="10"/>
-      <c r="P22" s="11"/>
-      <c r="Q22" s="14">
+      <c r="O22" s="11"/>
+      <c r="P22" s="14">
         <v>0.80139</v>
       </c>
+      <c r="Q22" s="10"/>
       <c r="R22" s="10"/>
       <c r="S22" s="10"/>
-      <c r="T22" s="10"/>
-      <c r="U22" s="11"/>
-      <c r="V22" s="14">
+      <c r="T22" s="11"/>
+      <c r="U22" s="14">
         <v>0.80139</v>
       </c>
+      <c r="V22" s="10"/>
       <c r="W22" s="10"/>
       <c r="X22" s="10"/>
-      <c r="Y22" s="10"/>
-      <c r="Z22" s="11"/>
-      <c r="AA22" s="14">
+      <c r="Y22" s="11"/>
+      <c r="Z22" s="14">
         <v>0.80139</v>
       </c>
+      <c r="AA22" s="10"/>
       <c r="AB22" s="10"/>
       <c r="AC22" s="10"/>
-      <c r="AD22" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="18.75">
-      <c r="A23" s="1"/>
-      <c r="B23" s="14">
+      <c r="A23" s="14">
         <v>0.85108</v>
       </c>
+      <c r="B23" s="10"/>
       <c r="C23" s="10"/>
       <c r="D23" s="10"/>
-      <c r="E23" s="10"/>
-      <c r="F23" s="11"/>
-      <c r="G23" s="14">
+      <c r="E23" s="11"/>
+      <c r="F23" s="14">
         <v>0.85108</v>
       </c>
+      <c r="G23" s="10"/>
       <c r="H23" s="10"/>
       <c r="I23" s="10"/>
-      <c r="J23" s="10"/>
-      <c r="K23" s="11"/>
-      <c r="L23" s="14">
+      <c r="J23" s="11"/>
+      <c r="K23" s="14">
         <v>0.85108</v>
       </c>
+      <c r="L23" s="10"/>
       <c r="M23" s="10"/>
       <c r="N23" s="10"/>
-      <c r="O23" s="10"/>
-      <c r="P23" s="11"/>
-      <c r="Q23" s="14">
+      <c r="O23" s="11"/>
+      <c r="P23" s="14">
         <v>0.85108</v>
       </c>
+      <c r="Q23" s="10"/>
       <c r="R23" s="10"/>
       <c r="S23" s="10"/>
-      <c r="T23" s="10"/>
-      <c r="U23" s="11"/>
-      <c r="V23" s="14">
+      <c r="T23" s="11"/>
+      <c r="U23" s="14">
         <v>0.85108</v>
       </c>
+      <c r="V23" s="10"/>
       <c r="W23" s="10"/>
       <c r="X23" s="10"/>
-      <c r="Y23" s="10"/>
-      <c r="Z23" s="11"/>
-      <c r="AA23" s="14">
+      <c r="Y23" s="11"/>
+      <c r="Z23" s="14">
         <v>0.85108</v>
       </c>
+      <c r="AA23" s="10"/>
       <c r="AB23" s="10"/>
       <c r="AC23" s="10"/>
-      <c r="AD23" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="18.75">
-      <c r="A24" s="1"/>
-      <c r="B24" s="14">
+      <c r="A24" s="14">
         <v>0.90339</v>
       </c>
+      <c r="B24" s="10"/>
       <c r="C24" s="10"/>
       <c r="D24" s="10"/>
-      <c r="E24" s="10"/>
-      <c r="F24" s="11"/>
-      <c r="G24" s="14">
+      <c r="E24" s="11"/>
+      <c r="F24" s="14">
         <v>0.90339</v>
       </c>
+      <c r="G24" s="10"/>
       <c r="H24" s="10"/>
       <c r="I24" s="10"/>
-      <c r="J24" s="10"/>
-      <c r="K24" s="11"/>
-      <c r="L24" s="14">
+      <c r="J24" s="11"/>
+      <c r="K24" s="14">
         <v>0.90339</v>
       </c>
+      <c r="L24" s="10"/>
       <c r="M24" s="10"/>
       <c r="N24" s="10"/>
-      <c r="O24" s="10"/>
-      <c r="P24" s="11"/>
-      <c r="Q24" s="14">
+      <c r="O24" s="11"/>
+      <c r="P24" s="14">
         <v>0.90339</v>
       </c>
+      <c r="Q24" s="10"/>
       <c r="R24" s="10"/>
       <c r="S24" s="10"/>
-      <c r="T24" s="10"/>
-      <c r="U24" s="11"/>
-      <c r="V24" s="14">
+      <c r="T24" s="11"/>
+      <c r="U24" s="14">
         <v>0.90339</v>
       </c>
+      <c r="V24" s="10"/>
       <c r="W24" s="10"/>
       <c r="X24" s="10"/>
-      <c r="Y24" s="10"/>
-      <c r="Z24" s="11"/>
-      <c r="AA24" s="14">
+      <c r="Y24" s="11"/>
+      <c r="Z24" s="14">
         <v>0.90339</v>
       </c>
+      <c r="AA24" s="10"/>
       <c r="AB24" s="10"/>
       <c r="AC24" s="10"/>
-      <c r="AD24" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="18.75">
-      <c r="A25" s="1"/>
-      <c r="B25" s="14">
+      <c r="A25" s="14">
         <v>0.95085</v>
       </c>
+      <c r="B25" s="10"/>
       <c r="C25" s="10"/>
       <c r="D25" s="10"/>
-      <c r="E25" s="10"/>
-      <c r="F25" s="11"/>
-      <c r="G25" s="14">
+      <c r="E25" s="11"/>
+      <c r="F25" s="14">
         <v>0.95085</v>
       </c>
+      <c r="G25" s="10"/>
       <c r="H25" s="10"/>
       <c r="I25" s="10"/>
-      <c r="J25" s="10"/>
-      <c r="K25" s="11"/>
-      <c r="L25" s="14">
+      <c r="J25" s="11"/>
+      <c r="K25" s="14">
         <v>0.95085</v>
       </c>
+      <c r="L25" s="10"/>
       <c r="M25" s="10"/>
       <c r="N25" s="10"/>
-      <c r="O25" s="10"/>
-      <c r="P25" s="11"/>
-      <c r="Q25" s="14">
+      <c r="O25" s="11"/>
+      <c r="P25" s="14">
         <v>0.95085</v>
       </c>
+      <c r="Q25" s="10"/>
       <c r="R25" s="10"/>
       <c r="S25" s="10"/>
-      <c r="T25" s="10"/>
-      <c r="U25" s="11"/>
-      <c r="V25" s="14">
+      <c r="T25" s="11"/>
+      <c r="U25" s="14">
         <v>0.95085</v>
       </c>
+      <c r="V25" s="10"/>
       <c r="W25" s="10"/>
       <c r="X25" s="10"/>
-      <c r="Y25" s="10"/>
-      <c r="Z25" s="11"/>
-      <c r="AA25" s="14">
+      <c r="Y25" s="11"/>
+      <c r="Z25" s="14">
         <v>0.95085</v>
       </c>
+      <c r="AA25" s="10"/>
       <c r="AB25" s="10"/>
       <c r="AC25" s="10"/>
-      <c r="AD25" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="18.75">
-      <c r="A26" s="1"/>
-      <c r="B26" s="9">
+      <c r="A26" s="9">
         <v>1</v>
       </c>
+      <c r="B26" s="10"/>
       <c r="C26" s="10"/>
       <c r="D26" s="10"/>
-      <c r="E26" s="10"/>
-      <c r="F26" s="11"/>
-      <c r="G26" s="9">
+      <c r="E26" s="11"/>
+      <c r="F26" s="9">
         <v>1</v>
       </c>
+      <c r="G26" s="10"/>
       <c r="H26" s="10"/>
       <c r="I26" s="10"/>
-      <c r="J26" s="10"/>
-      <c r="K26" s="11"/>
-      <c r="L26" s="9">
+      <c r="J26" s="11"/>
+      <c r="K26" s="9">
         <v>1</v>
       </c>
+      <c r="L26" s="10"/>
       <c r="M26" s="10"/>
       <c r="N26" s="10"/>
-      <c r="O26" s="10"/>
-      <c r="P26" s="11"/>
-      <c r="Q26" s="9">
+      <c r="O26" s="11"/>
+      <c r="P26" s="9">
         <v>1</v>
       </c>
+      <c r="Q26" s="10"/>
       <c r="R26" s="10"/>
       <c r="S26" s="10"/>
-      <c r="T26" s="10"/>
-      <c r="U26" s="11"/>
-      <c r="V26" s="9">
+      <c r="T26" s="11"/>
+      <c r="U26" s="9">
         <v>1</v>
       </c>
+      <c r="V26" s="10"/>
       <c r="W26" s="10"/>
       <c r="X26" s="10"/>
-      <c r="Y26" s="10"/>
-      <c r="Z26" s="11"/>
-      <c r="AA26" s="9">
+      <c r="Y26" s="11"/>
+      <c r="Z26" s="9">
         <v>1</v>
       </c>
+      <c r="AA26" s="10"/>
       <c r="AB26" s="10"/>
       <c r="AC26" s="10"/>
-      <c r="AD26" s="10"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>